<commit_message>
feature/fsel-5567: Update Export File
</commit_message>
<xml_diff>
--- a/Services/Fsel.System/Fsel.System.Api/Resources/ManagerReports/BaoCaoChuyenCan.xlsx
+++ b/Services/Fsel.System/Fsel.System.Api/Resources/ManagerReports/BaoCaoChuyenCan.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.System\Fsel.System.Api\Resources\ManagerReports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{345161E2-7FAD-47E8-B1BC-8A58A04621EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B1452C6-4775-4E72-85FD-633D32C29CAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7FD84967-D379-4295-B365-C4BAD0C1800B}"/>
   </bookViews>
@@ -27,9 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
-    <t>BÁO CÁO CHUYÊN CẦN (Academic &amp; Ielts)</t>
-  </si>
-  <si>
     <t>Trường</t>
   </si>
   <si>
@@ -109,6 +106,9 @@
   </si>
   <si>
     <t>Số điện thoại</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BÁO CÁO CHUYÊN CẦN </t>
   </si>
 </sst>
 </file>
@@ -620,7 +620,7 @@
   <sheetData>
     <row r="1" spans="1:15" ht="26.25" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="8" t="s">
-        <v>0</v>
+        <v>27</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -639,49 +639,49 @@
     </row>
     <row r="2" spans="1:15" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
       <c r="D2" s="10"/>
       <c r="E2" s="10"/>
       <c r="F2" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" s="1"/>
       <c r="H2" s="6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N2" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="O2" s="2"/>
     </row>
     <row r="3" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1"/>
       <c r="C3" s="1"/>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
       <c r="F3" s="1">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
@@ -695,14 +695,14 @@
     </row>
     <row r="4" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
       <c r="F4" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
@@ -716,14 +716,14 @@
     </row>
     <row r="5" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G5" s="11"/>
       <c r="H5" s="11"/>
@@ -737,49 +737,49 @@
     </row>
     <row r="6" spans="1:15" ht="30" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="I6" s="4" t="s">
+      <c r="J6" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="J6" s="4" t="s">
+      <c r="K6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="K6" s="4" t="s">
+      <c r="L6" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="L6" s="4" t="s">
+      <c r="M6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="N6" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="M6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="N6" s="4" t="s">
+      <c r="O6" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="O6" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>